<commit_message>
in progress api excel and form done working on airway bill
</commit_message>
<xml_diff>
--- a/public/file/Trax Book Corporate Shipment Template.xlsx
+++ b/public/file/Trax Book Corporate Shipment Template.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22827"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sonic\public\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7D84E1-578C-41A3-B1CB-AACBC35DB134}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8496"/>
+    <workbookView xWindow="-108" yWindow="372" windowWidth="23256" windowHeight="12696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Consignee Name</t>
   </si>
@@ -102,12 +103,15 @@
   </si>
   <si>
     <t>Delivery Type ID</t>
+  </si>
+  <si>
+    <t>Pieces</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -453,8 +457,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -481,10 +485,11 @@
     <col min="23" max="23" width="17.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="16.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="18" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -562,6 +567,9 @@
       </c>
       <c r="Z1" s="1" t="s">
         <v>24</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>